<commit_message>
Add collection step to DEAP flow evaluation
</commit_message>
<xml_diff>
--- a/交接文档/交接文档/04_评测集/医检证据助手-连续流程评测集.xlsx
+++ b/交接文档/交接文档/04_评测集/医检证据助手-连续流程评测集.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测数据" sheetId="1" r:id="R9ce3b62876ab4a5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="R93910fd676024baf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测数据" sheetId="1" r:id="R1b0006ebfaaa47e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="Rea38248e8d124fc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -567,7 +567,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C3" s="8" t="str">
-        <x:v>用户补充资料</x:v>
+        <x:v>用户补充基础信息</x:v>
       </x:c>
       <x:c r="D3" s="8" t="str">
         <x:v>否</x:v>
@@ -586,37 +586,56 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="130" customHeight="1">
-      <x:c r="A4" s="10" t="str">
+      <x:c r="A4" s="7" t="str">
         <x:v>F01</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="n">
+      <x:c r="B4" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="C4" s="11" t="str">
+      <x:c r="C4" s="8" t="str">
+        <x:v>继续收集检查资料</x:v>
+      </x:c>
+      <x:c r="D4" s="8" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>没有做过肝功能，也不清楚乙肝、丙肝检查结果。以前没有同部位影像资料。</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="str">
+        <x:v>继续只提出 1 条最关键补充确认，例如是否有腹痛、发热、黄疸、消化不适等相关症状，或是否有医生已给出的说明；不能直接生成最终资料包，除非用户明确要求。</x:v>
+      </x:c>
+      <x:c r="G4" s="8" t="str">
+        <x:v>在生成最终展示前保留追问空间；只追问 1 条；按知识库继续收集；不下诊断。</x:v>
+      </x:c>
+      <x:c r="H4" s="9" t="str">
+        <x:v>继续收集,症状确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="130" customHeight="1">
+      <x:c r="A5" s="10" t="str">
+        <x:v>F01</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
         <x:v>生成最终展示</x:v>
       </x:c>
-      <x:c r="D4" s="11" t="str">
+      <x:c r="D5" s="11" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="E4" s="11" t="str">
-        <x:v>先到这里，请生成患者易懂版病程梳理和医生查看版资料包。</x:v>
-      </x:c>
-      <x:c r="F4" s="11" t="str">
+      <x:c r="E5" s="11" t="str">
+        <x:v>没有腹痛、发热、黄疸或消化不适。先到这里，请生成患者易懂版病程梳理和医生查看版资料包。</x:v>
+      </x:c>
+      <x:c r="F5" s="11" t="str">
         <x:v>输出患者易懂版病程梳理和医生查看版资料包；包含资料来源、病程时间线、已知资料、仍缺资料、建议向医生确认的问题和安全声明；不输出原文依据、内部分类、命中规则或引用文档。</x:v>
       </x:c>
-      <x:c r="G4" s="11" t="str">
+      <x:c r="G5" s="11" t="str">
         <x:v>结构完整；表达简洁；不下诊断；不出现穿刺、手术、用药、复查周期建议；仍缺资料不能写成必须检查。</x:v>
       </x:c>
-      <x:c r="H4" s="12" t="str">
+      <x:c r="H5" s="12" t="str">
         <x:v>病程梳理,医生查看版资料包</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="130" customHeight="1">
-      <x:c r="A5"/>
-      <x:c r="B5"/>
-      <x:c r="C5"/>
-      <x:c r="D5"/>
-      <x:c r="E5"/>
     </x:row>
     <x:row r="6" ht="130" customHeight="1">
       <x:c r="A6"/>
@@ -651,27 +670,32 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>1. 这是三步连续流程评测，不要逐条刷新会话。</x:v>
+        <x:v>1. 这是四步连续流程评测，不要逐条刷新会话。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>2. 第 1 步刷新 chat 并上传测试图片；第 2、3 步在同一会话里继续发送。</x:v>
+        <x:v>2. 第 1 步刷新 chat 并上传测试图片；第 2、3、4 步在同一会话里继续发送。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="3" t="str">
-        <x:v>3. 重点观察：是否只追问 1 条、是否按知识库缺口追问、是否去掉测试字段。</x:v>
+        <x:v>3. 第 3 步是新增的信息收集环节，用来观察 AI 是否继续按知识库追问。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="3" t="str">
-        <x:v>4. 用户刚上传或粘贴资料后，不应输出“整理信息如下”，只输出下一条补充确认。</x:v>
+        <x:v>4. 重点观察：是否只追问 1 条、是否按知识库缺口追问、是否去掉测试字段。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
-        <x:v>5. 测试优先使用脱敏真实数据；资料不够时找学长补，不要编造。</x:v>
+        <x:v>5. 用户刚上传或粘贴资料后，不应输出“整理信息如下”，只输出下一条补充确认。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="3" t="str">
+        <x:v>6. 测试优先使用脱敏真实数据；资料不够时找学长补，不要编造。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Revise patient-facing output sections
</commit_message>
<xml_diff>
--- a/交接文档/交接文档/04_评测集/医检证据助手-连续流程评测集.xlsx
+++ b/交接文档/交接文档/04_评测集/医检证据助手-连续流程评测集.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测数据" sheetId="1" r:id="R1b0006ebfaaa47e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="Rea38248e8d124fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评测数据" sheetId="1" r:id="R5aeb19de7042425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="2" r:id="Rb26290b094af4066"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -625,13 +625,13 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
-        <x:v>没有腹痛、发热、黄疸或消化不适。先到这里，请生成患者易懂版病程梳理和医生查看版资料包。</x:v>
+        <x:v>没有腹痛、发热、黄疸或消化不适。先到这里，请生成患者展示版和医生查看版资料包。</x:v>
       </x:c>
       <x:c r="F5" s="11" t="str">
-        <x:v>输出患者易懂版病程梳理和医生查看版资料包；包含资料来源、病程时间线、已知资料、仍缺资料、建议向医生确认的问题和安全声明；不输出原文依据、内部分类、命中规则或引用文档。</x:v>
+        <x:v>输出患者展示版和医生查看版资料包。患者展示版必须只包含三部分：患者病程理解、疾病关键词解释、建议问医生的问题；语言要通俗易懂、大白话，确保患者能看懂。医生查看版保留资料来源、病程时间线、已知资料、仍缺资料、建议向医生确认的问题和安全声明；不输出原文依据、内部分类、命中规则或引用文档。</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str">
-        <x:v>结构完整；表达简洁；不下诊断；不出现穿刺、手术、用药、复查周期建议；仍缺资料不能写成必须检查。</x:v>
+        <x:v>患者版三部分齐全；关键词解释只解释报告中出现的词；表达简洁易懂；不下诊断；不出现穿刺、手术、用药、复查周期建议；仍缺资料不能写成必须检查。</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
         <x:v>病程梳理,医生查看版资料包</x:v>

</xml_diff>